<commit_message>
small bug fix, simpler demo order
</commit_message>
<xml_diff>
--- a/Python/orders_from_order.xlsx
+++ b/Python/orders_from_order.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -626,94 +626,6 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>TEENSY 4.1 H</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Teensy 4.1, USB, with header</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>45.71</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>NKS 200 GR</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Mains cable with safety plug, grey, 1.8 m</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>3.04</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>DEBO RE 1CH HL</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Developer boards - Relay module, 1 channel, 5 V, high/low</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>2.02</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>LIM-P-82-70</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Temperature limiter, 70Â°C, NC, 250 V.</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>1.98</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
added support for Conrad
</commit_message>
<xml_diff>
--- a/Python/orders_from_order.xlsx
+++ b/Python/orders_from_order.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -426,7 +426,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Schäfter + Kirchhoff</t>
+          <t>Conrad</t>
         </is>
       </c>
     </row>
@@ -460,232 +460,81 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">60FC-4-M6.2-01 | Fiber Collimator, focusable, housing Ã˜ 12 mm -3.00%, Achromat </t>
+          <t>2557557-8J | VALUE USB 2.0 Kabel, USB A Male - Micro USB B Male, wit, 3 m</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Fiber Collimator, focusable, housing Ã˜ 12 mm -3.00%
-Achromat f'6.2 mm / NA 0.2 / AR 350 - 700 nm
-Inclined coupling axis, FC-APC connection</t>
+          <t>VALUE USB 2.0 Kabel, USB A Male - Micro USB B Male, wit, 3 m</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>428.9256</t>
+          <t>2.8843</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>60FC-4-M6.2-01</t>
+          <t>2557557-8J</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>60FC-4-M8-10 | Fiber Collimator, focusable, housing Ã˜ 12 mm -3.00%, Monochromat</t>
+          <t>2269230-8J | PJRC Teensy41 Microcontroller Teensy 4.1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Fiber Collimator, focusable, housing Ã˜ 12 mm -3.00%
-Monochromat f'8 mm / NA 0.23 / AR 630 - 1080 nm
-Inclined coupling axis, FC-APC connection</t>
+          <t>PJRC Teensy41 Microcontroller Teensy 4.1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>315.7025</t>
+          <t>36.3554</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>60FC-4-M8-10</t>
+          <t>2269230-8J</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PMC-780-3-18E-500 | Old product code:, PMC-E-780-5.3-NA012-3-APC.EC-500-P, Singl</t>
+          <t>2445488-8J | Sygonix SY-4890976 Stekkerdoos 3-voudig Wit Randaarde stekker 1 stu</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Old product code:
-PMC-E-780-5.3-NA012-3-APC.EC-500-P
-Single-mode fiber cable, 5.0 m long</t>
+          <t>Sygonix SY-4890976 Stekkerdoos 3-voudig Wit Randaarde stekker 1 stuk(s)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>2.8843</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>PMC-780-3-18E-500</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>PMC-780-3-18-500 | Old product code: -3.00%, PMC-780-5.3-NA012-3-APC-500-P, Sing</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Old product code: -3.00%
-PMC-780-5.3-NA012-3-APC-500-P
-Single-mode fiber cable, 5.0 m long</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>427.2727</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>PMC-780-3-18-500</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>PMC-980-3-18E-500 | Old product code:, PMC-E-980-6.6-NA012-3-APC.EC-500-P, Singl</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Old product code:
-PMC-E-980-6.6-NA012-3-APC.EC-500-P
-Single-mode fiber cable, 5.0 m long</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>595.8678</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>PMC-980-3-18E-500</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>PMC-460-3-18-500 | Old product code:, PMC-460-3.3-NA012-3-APC-500-P, Single-mode</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Old product code:
-PMC-460-3.3-NA012-3-APC-500-P
-Single-mode fiber cable, 5.0 m long</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>468.595</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>PMC-460-3-18-500</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">60FC-4-A6.2S-02 | Fiber Collimator, focusable, housing Ã˜ 12 mm -3.00%, Asphere </t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Fiber Collimator, focusable, housing Ã˜ 12 mm -3.00%
-Asphere f'6.2 mm / NA 0.3 / AR 600 - 1100 nm
-Inclined coupling axis, FC-APC connection</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>219.0083</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>60FC-4-A6.2S-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">60FC-4-A6.2S-01 | Fiber Collimator, focusable, housing Ã˜ 12 mm -3.00%, Asphere </t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Fiber Collimator, focusable, housing Ã˜ 12 mm -3.00%
-Asphere f'6.2 mm / NA 0.3 / AR 350 - 700 nm
-Inclined coupling axis, FC-APC connection</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>371.9008</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>60FC-4-A6.2S-01</t>
+          <t>2445488-8J</t>
         </is>
       </c>
     </row>

</xml_diff>